<commit_message>
Update latest quarterly debt report PDF and public debt data export
</commit_message>
<xml_diff>
--- a/docs/kenya_public_debt_data.xlsx
+++ b/docs/kenya_public_debt_data.xlsx
@@ -79,7 +79,7 @@
     <t xml:space="preserve">Kenya Public Debt -- Notes &amp; Sources</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated: 12 September 2026, 17:20 UTC</t>
+    <t xml:space="preserve">Generated: 12 September 2026, 18:13 UTC</t>
   </si>
   <si>
     <t xml:space="preserve">Report: IEA Kenya Quarterly Macro &amp; Public Debt Report</t>
@@ -548,13 +548,13 @@
         <v>6</v>
       </c>
       <c r="B5" s="4" t="n">
-        <v>7395.43</v>
+        <v>7395.49</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>5674.77</v>
+        <v>5674.82</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>13070.2</v>
+        <v>13070.3</v>
       </c>
     </row>
     <row r="6">
@@ -576,13 +576,13 @@
         <v>8</v>
       </c>
       <c r="B7" s="4" t="n">
-        <v>135925</v>
+        <v>135926</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>104300</v>
+        <v>104301</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>240225</v>
+        <v>240226</v>
       </c>
     </row>
     <row r="8">
@@ -717,13 +717,13 @@
         <v>46277</v>
       </c>
       <c r="B3" t="n">
-        <v>7395.43</v>
+        <v>7395.49</v>
       </c>
       <c r="C3" t="n">
-        <v>5674.77</v>
+        <v>5674.82</v>
       </c>
       <c r="D3" t="n">
-        <v>13070.2</v>
+        <v>13070.3</v>
       </c>
       <c r="E3" t="n">
         <v>57</v>
@@ -735,13 +735,13 @@
         <v>100</v>
       </c>
       <c r="H3" t="n">
-        <v>135925</v>
+        <v>135926</v>
       </c>
       <c r="I3" t="n">
-        <v>104300</v>
+        <v>104301</v>
       </c>
       <c r="J3" t="n">
-        <v>240225</v>
+        <v>240226</v>
       </c>
       <c r="K3" t="n">
         <v>40</v>
@@ -758,13 +758,13 @@
         <v>46266</v>
       </c>
       <c r="B4" t="n">
-        <v>7387.78575342466</v>
+        <v>7387.83671232877</v>
       </c>
       <c r="C4" t="n">
-        <v>5668.79232876712</v>
+        <v>5668.83479452055</v>
       </c>
       <c r="D4" t="n">
-        <v>13039.538630137</v>
+        <v>13039.6235616438</v>
       </c>
       <c r="E4" t="n">
         <v>57</v>
@@ -776,13 +776,13 @@
         <v>100</v>
       </c>
       <c r="H4" t="n">
-        <v>135607</v>
+        <v>135608</v>
       </c>
       <c r="I4" t="n">
-        <v>104054</v>
+        <v>104055</v>
       </c>
       <c r="J4" t="n">
-        <v>239661</v>
+        <v>239663</v>
       </c>
       <c r="K4" t="n">
         <v>40</v>
@@ -799,13 +799,13 @@
         <v>46235</v>
       </c>
       <c r="B5" t="n">
-        <v>7366.24287671233</v>
+        <v>7366.26835616438</v>
       </c>
       <c r="C5" t="n">
-        <v>5651.94616438356</v>
+        <v>5651.96739726027</v>
       </c>
       <c r="D5" t="n">
-        <v>12953.1293150685</v>
+        <v>12953.1717808219</v>
       </c>
       <c r="E5" t="n">
         <v>57</v>
@@ -899,7 +899,7 @@
         <v>100</v>
       </c>
       <c r="H7" t="n">
-        <v>134140</v>
+        <v>134139</v>
       </c>
       <c r="I7" t="n">
         <v>102927</v>

</xml_diff>